<commit_message>
fix(exportacao): modelos oficiais da Plumene TB 2 e TB 3 com os precos arrumados pela fabrica (04/09)
Arquivos "PEDIDO PLU 2/3 2027 OFICIAL.xlsx" novos, byte a byte. TB 1 nao mudou.
Reproduzido com os 10 pedidos reais: 0 avisos. Na Plan2 ainda ficam 2206 e
22161 diferentes do PDF da tabela (TB 2 e TB 3) - avisado ao Yan; o app segue
gravando o preco do banco na celula.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/web/public/modelos/pedido-cs-2.xlsx
+++ b/apps/web/public/modelos/pedido-cs-2.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12210"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11910"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="2" r:id="rId1"/>
@@ -2877,9 +2877,7 @@
       <c r="AG12" s="77"/>
     </row>
     <row r="13" spans="1:33" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="93">
-        <v>22238</v>
-      </c>
+      <c r="A13" s="93"/>
       <c r="B13" s="98"/>
       <c r="C13" s="98"/>
       <c r="D13" s="98"/>
@@ -2891,18 +2889,10 @@
       <c r="J13" s="98"/>
       <c r="K13" s="98"/>
       <c r="L13" s="44"/>
-      <c r="M13" s="44">
-        <v>2</v>
-      </c>
-      <c r="N13" s="36">
-        <v>3</v>
-      </c>
-      <c r="O13" s="36">
-        <v>2</v>
-      </c>
-      <c r="P13" s="36">
-        <v>2</v>
-      </c>
+      <c r="M13" s="44"/>
+      <c r="N13" s="36"/>
+      <c r="O13" s="36"/>
+      <c r="P13" s="36"/>
       <c r="Q13" s="36"/>
       <c r="R13" s="36"/>
       <c r="S13" s="36"/>
@@ -2914,15 +2904,15 @@
       <c r="Y13" s="45"/>
       <c r="Z13" s="46">
         <f t="shared" ref="Z13:Z44" si="0">L13+M13+N13+O13+P13+U13+V13+W13+X13+Q13+R13+S13+T13</f>
-        <v>9</v>
-      </c>
-      <c r="AA13" s="27">
+        <v>0</v>
+      </c>
+      <c r="AA13" s="27" t="str">
         <f>IFERROR(VLOOKUP(A13,Plan2!$A$1:$F$777,6,0),"-")</f>
-        <v>63.9</v>
-      </c>
-      <c r="AB13" s="43">
+        <v>-</v>
+      </c>
+      <c r="AB13" s="43" t="str">
         <f>IFERROR(AA13*Z13,"-")</f>
-        <v>575.1</v>
+        <v>-</v>
       </c>
       <c r="AE13" s="17"/>
       <c r="AF13" s="7" t="s">
@@ -2931,9 +2921,7 @@
       <c r="AG13" s="33"/>
     </row>
     <row r="14" spans="1:33" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="94">
-        <v>22126</v>
-      </c>
+      <c r="A14" s="94"/>
       <c r="B14" s="98"/>
       <c r="C14" s="98"/>
       <c r="D14" s="98"/>
@@ -2945,15 +2933,9 @@
       <c r="J14" s="98"/>
       <c r="K14" s="98"/>
       <c r="L14" s="44"/>
-      <c r="M14" s="47">
-        <v>2</v>
-      </c>
-      <c r="N14" s="38">
-        <v>3</v>
-      </c>
-      <c r="O14" s="38">
-        <v>2</v>
-      </c>
+      <c r="M14" s="47"/>
+      <c r="N14" s="38"/>
+      <c r="O14" s="38"/>
       <c r="P14" s="38"/>
       <c r="Q14" s="38"/>
       <c r="R14" s="38"/>
@@ -2966,15 +2948,15 @@
       <c r="Y14" s="40"/>
       <c r="Z14" s="41">
         <f t="shared" si="0"/>
-        <v>7</v>
-      </c>
-      <c r="AA14" s="42">
+        <v>0</v>
+      </c>
+      <c r="AA14" s="42" t="str">
         <f>IFERROR(VLOOKUP(A14,Plan2!$A$1:$F$777,6,0),"-")</f>
-        <v>64.900000000000006</v>
-      </c>
-      <c r="AB14" s="43">
+        <v>-</v>
+      </c>
+      <c r="AB14" s="43" t="str">
         <f>IFERROR(AA14*Z14,"-")</f>
-        <v>454.30000000000007</v>
+        <v>-</v>
       </c>
       <c r="AF14" s="7">
         <v>87</v>
@@ -2982,9 +2964,7 @@
       <c r="AG14" s="33"/>
     </row>
     <row r="15" spans="1:33" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="95">
-        <v>22128</v>
-      </c>
+      <c r="A15" s="95"/>
       <c r="B15" s="98"/>
       <c r="C15" s="98"/>
       <c r="D15" s="98"/>
@@ -2996,18 +2976,10 @@
       <c r="J15" s="98"/>
       <c r="K15" s="98"/>
       <c r="L15" s="44"/>
-      <c r="M15" s="48">
-        <v>2</v>
-      </c>
-      <c r="N15" s="36">
-        <v>3</v>
-      </c>
-      <c r="O15" s="36">
-        <v>2</v>
-      </c>
-      <c r="P15" s="36">
-        <v>2</v>
-      </c>
+      <c r="M15" s="48"/>
+      <c r="N15" s="36"/>
+      <c r="O15" s="36"/>
+      <c r="P15" s="36"/>
       <c r="Q15" s="36"/>
       <c r="R15" s="36"/>
       <c r="S15" s="36"/>
@@ -3019,15 +2991,15 @@
       <c r="Y15" s="26"/>
       <c r="Z15" s="32">
         <f t="shared" si="0"/>
-        <v>9</v>
-      </c>
-      <c r="AA15" s="27">
+        <v>0</v>
+      </c>
+      <c r="AA15" s="27" t="str">
         <f>IFERROR(VLOOKUP(A15,Plan2!$A$1:$F$777,6,0),"-")</f>
-        <v>60.9</v>
-      </c>
-      <c r="AB15" s="28">
+        <v>-</v>
+      </c>
+      <c r="AB15" s="28" t="str">
         <f t="shared" ref="AB15:AB44" si="1">IFERROR(AA15*Z15,"-")</f>
-        <v>548.1</v>
+        <v>-</v>
       </c>
       <c r="AF15" s="8" t="s">
         <v>53</v>
@@ -3035,9 +3007,7 @@
       <c r="AG15" s="33"/>
     </row>
     <row r="16" spans="1:33" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="95">
-        <v>22243</v>
-      </c>
+      <c r="A16" s="95"/>
       <c r="B16" s="98"/>
       <c r="C16" s="98"/>
       <c r="D16" s="98"/>
@@ -3049,18 +3019,10 @@
       <c r="J16" s="98"/>
       <c r="K16" s="98"/>
       <c r="L16" s="44"/>
-      <c r="M16" s="48">
-        <v>2</v>
-      </c>
-      <c r="N16" s="36">
-        <v>3</v>
-      </c>
-      <c r="O16" s="36">
-        <v>2</v>
-      </c>
-      <c r="P16" s="36">
-        <v>2</v>
-      </c>
+      <c r="M16" s="48"/>
+      <c r="N16" s="36"/>
+      <c r="O16" s="36"/>
+      <c r="P16" s="36"/>
       <c r="Q16" s="36"/>
       <c r="R16" s="36"/>
       <c r="S16" s="36"/>
@@ -3072,15 +3034,15 @@
       <c r="Y16" s="26"/>
       <c r="Z16" s="32">
         <f t="shared" si="0"/>
-        <v>9</v>
-      </c>
-      <c r="AA16" s="27">
+        <v>0</v>
+      </c>
+      <c r="AA16" s="27" t="str">
         <f>IFERROR(VLOOKUP(A16,Plan2!$A$1:$F$777,6,0),"-")</f>
-        <v>60.9</v>
-      </c>
-      <c r="AB16" s="28">
+        <v>-</v>
+      </c>
+      <c r="AB16" s="28" t="str">
         <f t="shared" si="1"/>
-        <v>548.1</v>
+        <v>-</v>
       </c>
       <c r="AF16" s="7">
         <v>88</v>
@@ -3088,9 +3050,7 @@
       <c r="AG16" s="33"/>
     </row>
     <row r="17" spans="1:33" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="95">
-        <v>2213</v>
-      </c>
+      <c r="A17" s="95"/>
       <c r="B17" s="98"/>
       <c r="C17" s="98"/>
       <c r="D17" s="98"/>
@@ -3102,18 +3062,10 @@
       <c r="J17" s="98"/>
       <c r="K17" s="98"/>
       <c r="L17" s="44"/>
-      <c r="M17" s="48">
-        <v>1</v>
-      </c>
-      <c r="N17" s="36">
-        <v>1</v>
-      </c>
-      <c r="O17" s="36">
-        <v>1</v>
-      </c>
-      <c r="P17" s="36">
-        <v>1</v>
-      </c>
+      <c r="M17" s="48"/>
+      <c r="N17" s="36"/>
+      <c r="O17" s="36"/>
+      <c r="P17" s="36"/>
       <c r="Q17" s="36"/>
       <c r="R17" s="36"/>
       <c r="S17" s="36"/>
@@ -3125,15 +3077,15 @@
       <c r="Y17" s="26"/>
       <c r="Z17" s="32">
         <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
-      <c r="AA17" s="27">
+        <v>0</v>
+      </c>
+      <c r="AA17" s="27" t="str">
         <f>IFERROR(VLOOKUP(A17,Plan2!$A$1:$F$777,6,0),"-")</f>
-        <v>65.900000000000006</v>
-      </c>
-      <c r="AB17" s="28">
+        <v>-</v>
+      </c>
+      <c r="AB17" s="28" t="str">
         <f t="shared" si="1"/>
-        <v>263.60000000000002</v>
+        <v>-</v>
       </c>
       <c r="AF17" s="7" t="s">
         <v>54</v>
@@ -3141,9 +3093,7 @@
       <c r="AG17" s="33"/>
     </row>
     <row r="18" spans="1:33" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="95">
-        <v>2279</v>
-      </c>
+      <c r="A18" s="95"/>
       <c r="B18" s="98"/>
       <c r="C18" s="98"/>
       <c r="D18" s="98"/>
@@ -3156,15 +3106,9 @@
       <c r="K18" s="98"/>
       <c r="L18" s="44"/>
       <c r="M18" s="48"/>
-      <c r="N18" s="36">
-        <v>2</v>
-      </c>
-      <c r="O18" s="36">
-        <v>2</v>
-      </c>
-      <c r="P18" s="36">
-        <v>2</v>
-      </c>
+      <c r="N18" s="36"/>
+      <c r="O18" s="36"/>
+      <c r="P18" s="36"/>
       <c r="Q18" s="36"/>
       <c r="R18" s="36"/>
       <c r="S18" s="36"/>
@@ -3176,15 +3120,15 @@
       <c r="Y18" s="26"/>
       <c r="Z18" s="32">
         <f t="shared" si="0"/>
-        <v>6</v>
-      </c>
-      <c r="AA18" s="27">
+        <v>0</v>
+      </c>
+      <c r="AA18" s="27" t="str">
         <f>IFERROR(VLOOKUP(A18,Plan2!$A$1:$F$777,6,0),"-")</f>
-        <v>72.900000000000006</v>
-      </c>
-      <c r="AB18" s="28">
+        <v>-</v>
+      </c>
+      <c r="AB18" s="28" t="str">
         <f t="shared" si="1"/>
-        <v>437.40000000000003</v>
+        <v>-</v>
       </c>
       <c r="AF18" s="7">
         <v>90</v>
@@ -3192,9 +3136,7 @@
       <c r="AG18" s="33"/>
     </row>
     <row r="19" spans="1:33" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="95">
-        <v>2215</v>
-      </c>
+      <c r="A19" s="95"/>
       <c r="B19" s="98"/>
       <c r="C19" s="98"/>
       <c r="D19" s="98"/>
@@ -3207,15 +3149,9 @@
       <c r="K19" s="98"/>
       <c r="L19" s="44"/>
       <c r="M19" s="48"/>
-      <c r="N19" s="36">
-        <v>1</v>
-      </c>
-      <c r="O19" s="36">
-        <v>2</v>
-      </c>
-      <c r="P19" s="36">
-        <v>1</v>
-      </c>
+      <c r="N19" s="36"/>
+      <c r="O19" s="36"/>
+      <c r="P19" s="36"/>
       <c r="Q19" s="36"/>
       <c r="R19" s="36"/>
       <c r="S19" s="36"/>
@@ -3227,15 +3163,15 @@
       <c r="Y19" s="26"/>
       <c r="Z19" s="32">
         <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
-      <c r="AA19" s="27">
+        <v>0</v>
+      </c>
+      <c r="AA19" s="27" t="str">
         <f>IFERROR(VLOOKUP(A19,Plan2!$A$1:$F$777,6,0),"-")</f>
-        <v>78</v>
-      </c>
-      <c r="AB19" s="28">
+        <v>-</v>
+      </c>
+      <c r="AB19" s="28" t="str">
         <f t="shared" si="1"/>
-        <v>312</v>
+        <v>-</v>
       </c>
       <c r="AF19" s="7" t="s">
         <v>55</v>
@@ -3243,9 +3179,7 @@
       <c r="AG19" s="33"/>
     </row>
     <row r="20" spans="1:33" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="95">
-        <v>2230</v>
-      </c>
+      <c r="A20" s="95"/>
       <c r="B20" s="98"/>
       <c r="C20" s="98"/>
       <c r="D20" s="98"/>
@@ -3257,18 +3191,10 @@
       <c r="J20" s="98"/>
       <c r="K20" s="98"/>
       <c r="L20" s="44"/>
-      <c r="M20" s="48">
-        <v>2</v>
-      </c>
-      <c r="N20" s="36">
-        <v>2</v>
-      </c>
-      <c r="O20" s="36">
-        <v>2</v>
-      </c>
-      <c r="P20" s="36">
-        <v>2</v>
-      </c>
+      <c r="M20" s="48"/>
+      <c r="N20" s="36"/>
+      <c r="O20" s="36"/>
+      <c r="P20" s="36"/>
       <c r="Q20" s="36"/>
       <c r="R20" s="36"/>
       <c r="S20" s="36"/>
@@ -3280,15 +3206,15 @@
       <c r="Y20" s="26"/>
       <c r="Z20" s="32">
         <f t="shared" si="0"/>
-        <v>8</v>
-      </c>
-      <c r="AA20" s="27">
+        <v>0</v>
+      </c>
+      <c r="AA20" s="27" t="str">
         <f>IFERROR(VLOOKUP(A20,Plan2!$A$1:$F$777,6,0),"-")</f>
-        <v>84.9</v>
-      </c>
-      <c r="AB20" s="28">
+        <v>-</v>
+      </c>
+      <c r="AB20" s="28" t="str">
         <f t="shared" si="1"/>
-        <v>679.2</v>
+        <v>-</v>
       </c>
       <c r="AF20" s="7">
         <v>91</v>
@@ -4359,14 +4285,14 @@
       <c r="Y45" s="30"/>
       <c r="Z45" s="31">
         <f>SUM(Z13:Z44)</f>
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="AA45" s="53" t="s">
         <v>148</v>
       </c>
       <c r="AB45" s="54">
         <f>SUM(AB13:AB44)</f>
-        <v>3817.8</v>
+        <v>0</v>
       </c>
       <c r="AC45" s="21"/>
       <c r="AF45" s="8">
@@ -4405,7 +4331,7 @@
         <v>149</v>
       </c>
       <c r="AB46" s="70">
-        <v>0.12</v>
+        <v>0</v>
       </c>
       <c r="AC46" s="55"/>
       <c r="AF46" s="8" t="s">
@@ -4445,7 +4371,7 @@
       </c>
       <c r="AB47" s="56">
         <f>AB45*AB46</f>
-        <v>458.13600000000002</v>
+        <v>0</v>
       </c>
       <c r="AC47" s="55"/>
       <c r="AF47" s="8">
@@ -4485,7 +4411,7 @@
       </c>
       <c r="AB48" s="139">
         <f>AB45-AB47</f>
-        <v>3359.6640000000002</v>
+        <v>0</v>
       </c>
       <c r="AC48" s="21"/>
       <c r="AF48" s="8" t="s">
@@ -7210,7 +7136,7 @@
       <c r="D78" s="34"/>
       <c r="E78" s="35"/>
       <c r="F78" s="88">
-        <v>133.9</v>
+        <v>134.9</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.2">
@@ -7234,7 +7160,7 @@
       <c r="D80" s="34"/>
       <c r="E80" s="35"/>
       <c r="F80" s="88">
-        <v>111.9</v>
+        <v>112.9</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.2">
@@ -7366,7 +7292,7 @@
       <c r="D91" s="34"/>
       <c r="E91" s="35"/>
       <c r="F91" s="88">
-        <v>98.8</v>
+        <v>98.9</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.2">
@@ -8196,7 +8122,7 @@
       <c r="D160" s="34"/>
       <c r="E160" s="35"/>
       <c r="F160" s="88">
-        <v>92.9</v>
+        <v>91.9</v>
       </c>
     </row>
     <row r="161" spans="1:6" x14ac:dyDescent="0.2">
@@ -8328,7 +8254,7 @@
       <c r="D171" s="34"/>
       <c r="E171" s="35"/>
       <c r="F171" s="88">
-        <v>59.9</v>
+        <v>60.9</v>
       </c>
     </row>
     <row r="172" spans="1:6" x14ac:dyDescent="0.2">
@@ -8340,7 +8266,7 @@
       <c r="D172" s="34"/>
       <c r="E172" s="35"/>
       <c r="F172" s="88">
-        <v>62.9</v>
+        <v>63.9</v>
       </c>
     </row>
     <row r="173" spans="1:6" x14ac:dyDescent="0.2">
@@ -8544,7 +8470,7 @@
       <c r="D189" s="34"/>
       <c r="E189" s="35"/>
       <c r="F189" s="88">
-        <v>60.5</v>
+        <v>60.9</v>
       </c>
     </row>
     <row r="190" spans="1:6" x14ac:dyDescent="0.2">
@@ -21881,7 +21807,7 @@
       <c r="F2784" s="91"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="3kEDw3lOXuwI7BvP7C4Zi5aItLxtd7US1hYJC8b14elQ1LmV6yHY3mHAJUMVqg/Q+PewRZknBQfTgTnwXhyGmA==" saltValue="drzZi0z8zr7Kjlwli5pRxg==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="PWSuG257p6n8lbhUwiF4tw0Pw118H58kN5D1kMLelOjlvh7tk+DHXUlR9/bt9DIwckwntPls3dJdsuZWT849lA==" saltValue="zLUyB87KH77CUOpfqGU80w==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <sortState ref="A2:B231">
     <sortCondition ref="A1"/>
   </sortState>

</xml_diff>